<commit_message>
updated project status tracker
</commit_message>
<xml_diff>
--- a/review/project_status_tracker_super_long_wave.xlsx
+++ b/review/project_status_tracker_super_long_wave.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yutak\eda\designs\03_super_long_wave\2026_sscs_gf180\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9A85684-BA3B-4BA5-B416-E8E8F4596ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC2D5275-B9E9-4E08-A669-7FC87596789B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="63">
   <si>
     <t>No</t>
     <phoneticPr fontId="1"/>
@@ -228,6 +228,41 @@
   <si>
     <t>Ongoing</t>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>gf180mcu_stdcells</t>
+  </si>
+  <si>
+    <t>opamp</t>
+  </si>
+  <si>
+    <t>current_mirror</t>
+  </si>
+  <si>
+    <t>scdac</t>
+  </si>
+  <si>
+    <t>sreg</t>
+  </si>
+  <si>
+    <t>sw_matrix</t>
+  </si>
+  <si>
+    <t>trans_gate</t>
+  </si>
+  <si>
+    <t>trans_gate</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>bmr</t>
+  </si>
+  <si>
+    <t>bmr</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>c4_all</t>
   </si>
 </sst>
 </file>
@@ -435,7 +470,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -483,6 +518,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
@@ -764,13 +800,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="5.75" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="18.125" customWidth="1"/>
-    <col min="4" max="4" width="14.75" customWidth="1"/>
+    <col min="4" max="4" width="18.75" customWidth="1"/>
     <col min="5" max="5" width="11.875" customWidth="1"/>
     <col min="6" max="6" width="10.625" customWidth="1"/>
     <col min="7" max="7" width="13.125" customWidth="1"/>
@@ -841,7 +877,9 @@
       <c r="C4" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="4"/>
+      <c r="D4" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="E4" s="10" t="s">
         <v>11</v>
       </c>
@@ -869,7 +907,9 @@
       <c r="C5" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D5" s="4"/>
+      <c r="D5" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="E5" s="10" t="s">
         <v>11</v>
       </c>
@@ -897,7 +937,9 @@
       <c r="C6" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="4"/>
+      <c r="D6" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="E6" s="10" t="s">
         <v>11</v>
       </c>
@@ -925,7 +967,9 @@
       <c r="C7" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="4"/>
+      <c r="D7" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="E7" s="10" t="s">
         <v>11</v>
       </c>
@@ -979,7 +1023,7 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="3">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>6</v>
@@ -1011,7 +1055,7 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="3">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>10</v>
@@ -1043,7 +1087,7 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="3">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="4" t="s">
@@ -1073,7 +1117,7 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="3">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>26</v>
@@ -1081,7 +1125,9 @@
       <c r="C12" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="4"/>
+      <c r="D12" s="16" t="s">
+        <v>53</v>
+      </c>
       <c r="E12" s="10" t="s">
         <v>11</v>
       </c>
@@ -1103,7 +1149,7 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="3">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>22</v>
@@ -1111,7 +1157,9 @@
       <c r="C13" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="4"/>
+      <c r="D13" s="16" t="s">
+        <v>54</v>
+      </c>
       <c r="E13" s="10" t="s">
         <v>11</v>
       </c>
@@ -1133,7 +1181,7 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="3">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>24</v>
@@ -1141,7 +1189,9 @@
       <c r="C14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="4"/>
+      <c r="D14" s="16" t="s">
+        <v>55</v>
+      </c>
       <c r="E14" s="10" t="s">
         <v>11</v>
       </c>
@@ -1163,13 +1213,15 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="3">
-        <v>14</v>
-      </c>
-      <c r="B15" s="9"/>
+        <v>12</v>
+      </c>
+      <c r="B15" s="11"/>
       <c r="C15" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="4"/>
+      <c r="D15" s="16" t="s">
+        <v>55</v>
+      </c>
       <c r="E15" s="10" t="s">
         <v>11</v>
       </c>
@@ -1191,45 +1243,43 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="3">
-        <v>15</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>46</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="B16" s="9"/>
       <c r="C16" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D16" s="4"/>
+        <v>61</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="E16" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="J16" s="6" t="s">
-        <v>50</v>
-      </c>
+      <c r="G16" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="3">
-        <v>18</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>25</v>
+        <v>14</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>46</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D17" s="4"/>
+        <v>42</v>
+      </c>
+      <c r="D17" s="16" t="s">
+        <v>56</v>
+      </c>
       <c r="E17" s="10" t="s">
         <v>11</v>
       </c>
@@ -1251,13 +1301,17 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="3">
-        <v>19</v>
-      </c>
-      <c r="B18" s="11"/>
+        <v>15</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>25</v>
+      </c>
       <c r="C18" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="4"/>
+        <v>31</v>
+      </c>
+      <c r="D18" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="E18" s="10" t="s">
         <v>11</v>
       </c>
@@ -1279,13 +1333,15 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="3">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B19" s="11"/>
       <c r="C19" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D19" s="4"/>
+        <v>28</v>
+      </c>
+      <c r="D19" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="E19" s="10" t="s">
         <v>11</v>
       </c>
@@ -1307,13 +1363,15 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="3">
-        <v>21</v>
-      </c>
-      <c r="B20" s="9"/>
+        <v>17</v>
+      </c>
+      <c r="B20" s="11"/>
       <c r="C20" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D20" s="4"/>
+        <v>29</v>
+      </c>
+      <c r="D20" s="16" t="s">
+        <v>57</v>
+      </c>
       <c r="E20" s="10" t="s">
         <v>11</v>
       </c>
@@ -1335,31 +1393,93 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="3">
-        <v>23</v>
-      </c>
-      <c r="B21" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" s="11"/>
+      <c r="C21" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10">
+      <c r="A22" s="3">
+        <v>19</v>
+      </c>
+      <c r="B22" s="9"/>
+      <c r="C22" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D22" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10">
+      <c r="A23" s="3">
+        <v>20</v>
+      </c>
+      <c r="B23" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C23" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="4"/>
-      <c r="E21" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F21" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G21" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="H21" s="5" t="s">
+      <c r="D23" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="H23" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="I21" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="J21" s="7" t="s">
+      <c r="I23" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J23" s="7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1370,6 +1490,20 @@
     <hyperlink ref="D9" r:id="rId2" xr:uid="{7EBF558B-AD84-48C4-BFD0-1B0FABBBDE93}"/>
     <hyperlink ref="D10" r:id="rId3" xr:uid="{71D7476D-A843-4F5E-9D30-F45859B20076}"/>
     <hyperlink ref="D11" r:id="rId4" xr:uid="{7566836C-A68A-46B1-92DD-C6EDA397B3DB}"/>
+    <hyperlink ref="D4" r:id="rId5" xr:uid="{7393101A-AB0A-4579-A972-F38C2C0EC13D}"/>
+    <hyperlink ref="D5:D7" r:id="rId6" display="gf180mcu_stdcells" xr:uid="{B9DE6BBC-0C69-4581-9249-E15DB0706FB4}"/>
+    <hyperlink ref="D12" r:id="rId7" xr:uid="{32280CC4-B8B0-4801-8042-3F259E8105B3}"/>
+    <hyperlink ref="D13" r:id="rId8" xr:uid="{C03EC173-0A90-4CFE-A545-060657B9C27D}"/>
+    <hyperlink ref="D14" r:id="rId9" xr:uid="{0D0DDB28-8942-43DD-834F-24F6CB67DF40}"/>
+    <hyperlink ref="D15" r:id="rId10" xr:uid="{FC2B0A46-C7C0-4FE4-8979-319B24915BCA}"/>
+    <hyperlink ref="D17" r:id="rId11" xr:uid="{DFD89CA2-3297-4298-B03D-55C8B623ABD0}"/>
+    <hyperlink ref="D18" r:id="rId12" xr:uid="{68F42C81-B341-4F88-8B82-EC45137B713A}"/>
+    <hyperlink ref="D19" r:id="rId13" xr:uid="{094BDAD3-A1C5-4C19-9C8D-107DFB2CA644}"/>
+    <hyperlink ref="D20" r:id="rId14" xr:uid="{75BB7E37-A25E-40CB-84D9-D881201AC00C}"/>
+    <hyperlink ref="D21" r:id="rId15" xr:uid="{D32F0983-8E06-499B-A5FC-5A07C4C61305}"/>
+    <hyperlink ref="D16" r:id="rId16" xr:uid="{DB6838D7-F735-4F3C-89CC-3FED158561A9}"/>
+    <hyperlink ref="D22" r:id="rId17" xr:uid="{DE0BC474-D7BF-4628-8E6C-E32B16E872E1}"/>
+    <hyperlink ref="D23" r:id="rId18" xr:uid="{E6411010-698F-4AEB-A056-0971ECB79120}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
changed name in pfd.gds
</commit_message>
<xml_diff>
--- a/review/project_status_tracker_super_long_wave.xlsx
+++ b/review/project_status_tracker_super_long_wave.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yutak\eda\designs\03_super_long_wave\2026_sscs_gf180\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC2D5275-B9E9-4E08-A669-7FC87596789B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9914EF1A-DEE9-4B9E-972D-2A87976EA4A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="2190" windowWidth="21600" windowHeight="14130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="status" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="64">
   <si>
     <t>No</t>
     <phoneticPr fontId="1"/>
@@ -263,6 +263,10 @@
   </si>
   <si>
     <t>c4_all</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -301,7 +305,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -326,6 +330,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -470,7 +480,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -519,6 +529,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
@@ -1014,11 +1027,11 @@
       <c r="H8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>13</v>
+      <c r="I8" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:10">

</xml_diff>

<commit_message>
project status tracker udpated
</commit_message>
<xml_diff>
--- a/review/project_status_tracker_super_long_wave.xlsx
+++ b/review/project_status_tracker_super_long_wave.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yutak\eda\designs\03_super_long_wave\2026_sscs_gf180\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51645144-5984-4F64-9671-51E1B177D7EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA9495DB-6D46-433B-893F-83FFC738FA12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="status" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="68">
   <si>
     <t>No</t>
     <phoneticPr fontId="1"/>
@@ -270,6 +281,18 @@
   </si>
   <si>
     <t>updated on Aug 3</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>GDS file is not created</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Green light to integrate. LVS and DRC passed.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>GDS file was created, LVS and/or DRS are not passed.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -484,7 +507,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -536,6 +559,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
@@ -817,7 +841,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="5.75" customWidth="1"/>
@@ -830,203 +854,115 @@
     <col min="8" max="8" width="10.625" customWidth="1"/>
     <col min="9" max="9" width="12.25" customWidth="1"/>
     <col min="10" max="11" width="7.25" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>7</v>
       </c>
+      <c r="H1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" t="s">
+      <c r="G2">
+        <f>COUNTIF(H8:H27,H2)</f>
+        <v>3</v>
+      </c>
+      <c r="H2" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="G3">
+        <f t="shared" ref="G3:G4" si="0">COUNTIF(H9:H28,H3)</f>
+        <v>5</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="G4">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="H4" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="25" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" t="s">
         <v>64</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E6" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="14"/>
-      <c r="G2" s="19" t="s">
+      <c r="F6" s="14"/>
+      <c r="G6" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="13"/>
-    </row>
-    <row r="3" spans="1:11" s="1" customFormat="1" ht="42" customHeight="1">
-      <c r="A3" s="2" t="s">
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="13"/>
+    </row>
+    <row r="7" spans="1:11" s="1" customFormat="1" ht="42" customHeight="1">
+      <c r="A7" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F7" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G7" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H7" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I7" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="J7" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="15" t="s">
+      <c r="K7" s="15" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="3">
-        <v>1</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="3">
-        <v>2</v>
-      </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="3">
-        <v>3</v>
-      </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
-      <c r="A7" s="3">
-        <v>4</v>
-      </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>17</v>
+        <v>37</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>50</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>11</v>
@@ -1035,68 +971,60 @@
         <v>12</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I8" s="6">
-        <v>1E-3</v>
-      </c>
-      <c r="J8" s="22" t="s">
-        <v>61</v>
+        <v>45</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6" t="s">
+        <v>45</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="3">
-        <v>6</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>6</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B9" s="11"/>
       <c r="C9" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>18</v>
+        <v>41</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>50</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F9" s="18" t="s">
         <v>12</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="6">
-        <v>1E-3</v>
-      </c>
+      <c r="I9" s="6"/>
       <c r="J9" s="6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="3">
-        <v>7</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>10</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B10" s="11"/>
       <c r="C10" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>19</v>
+        <v>39</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>50</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>11</v>
@@ -1105,31 +1033,29 @@
         <v>12</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I10" s="22">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="J10" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>13</v>
+        <v>45</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="3">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>20</v>
+        <v>38</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>50</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>11</v>
@@ -1138,33 +1064,31 @@
         <v>12</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I11" s="22">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="J11" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="K11" s="7" t="s">
-        <v>13</v>
+        <v>45</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="3">
-        <v>9</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>26</v>
+        <v>5</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>5</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>11</v>
@@ -1172,17 +1096,17 @@
       <c r="F12" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G12" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>12</v>
+      <c r="G12" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>49</v>
       </c>
       <c r="I12" s="6">
         <v>1E-3</v>
       </c>
-      <c r="J12" s="6" t="s">
-        <v>48</v>
+      <c r="J12" s="22" t="s">
+        <v>61</v>
       </c>
       <c r="K12" s="6" t="s">
         <v>48</v>
@@ -1190,51 +1114,51 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="3">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F13" s="18" t="s">
         <v>12</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="H13" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="K13" s="7" t="s">
-        <v>13</v>
+        <v>47</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I13" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="3">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>11</v>
@@ -1245,14 +1169,14 @@
       <c r="G14" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="H14" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="J14" s="7" t="s">
-        <v>13</v>
+      <c r="H14" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I14" s="22">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J14" s="22" t="s">
+        <v>61</v>
       </c>
       <c r="K14" s="7" t="s">
         <v>13</v>
@@ -1260,14 +1184,14 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="3">
-        <v>12</v>
-      </c>
-      <c r="B15" s="11"/>
+        <v>8</v>
+      </c>
+      <c r="B15" s="9"/>
       <c r="C15" s="4" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>11</v>
@@ -1278,14 +1202,14 @@
       <c r="G15" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="H15" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="I15" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="J15" s="7" t="s">
-        <v>13</v>
+      <c r="H15" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I15" s="22">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J15" s="22" t="s">
+        <v>61</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>13</v>
@@ -1293,14 +1217,16 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="3">
-        <v>13</v>
-      </c>
-      <c r="B16" s="9"/>
+        <v>9</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>26</v>
+      </c>
       <c r="C16" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>11</v>
@@ -1308,34 +1234,34 @@
       <c r="F16" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I16" s="22">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="J16" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="K16" s="7" t="s">
-        <v>13</v>
+      <c r="G16" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I16" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="3">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>11</v>
@@ -1343,34 +1269,34 @@
       <c r="F17" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G17" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I17" s="6">
-        <v>1E-3</v>
-      </c>
-      <c r="J17" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="K17" s="6" t="s">
-        <v>48</v>
+      <c r="G17" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="H17" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="3">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>11</v>
@@ -1378,32 +1304,32 @@
       <c r="F18" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G18" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I18" s="6">
-        <v>1E-3</v>
-      </c>
-      <c r="J18" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="K18" s="6" t="s">
-        <v>48</v>
+      <c r="G18" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="H18" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="3">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B19" s="11"/>
       <c r="C19" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>11</v>
@@ -1411,32 +1337,32 @@
       <c r="F19" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G19" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="H19" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I19" s="6">
-        <v>1E-3</v>
-      </c>
-      <c r="J19" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="K19" s="6" t="s">
-        <v>48</v>
+      <c r="G19" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="H19" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="3">
-        <v>17</v>
-      </c>
-      <c r="B20" s="11"/>
+        <v>13</v>
+      </c>
+      <c r="B20" s="9"/>
       <c r="C20" s="4" t="s">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>11</v>
@@ -1444,32 +1370,34 @@
       <c r="F20" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G20" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I20" s="6">
-        <v>1E-3</v>
-      </c>
-      <c r="J20" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="K20" s="6" t="s">
-        <v>48</v>
+      <c r="G20" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I20" s="22">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J20" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="3">
-        <v>18</v>
-      </c>
-      <c r="B21" s="11"/>
+        <v>14</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="C21" s="4" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>11</v>
@@ -1495,14 +1423,16 @@
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="3">
-        <v>19</v>
-      </c>
-      <c r="B22" s="9"/>
+        <v>15</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>25</v>
+      </c>
       <c r="C22" s="4" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>11</v>
@@ -1528,16 +1458,14 @@
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="3">
-        <v>20</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>36</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="B23" s="11"/>
       <c r="C23" s="4" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>11</v>
@@ -1548,40 +1476,174 @@
       <c r="G23" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="H23" s="5" t="s">
-        <v>49</v>
+      <c r="H23" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="I23" s="6">
         <v>1E-3</v>
       </c>
-      <c r="J23" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="K23" s="7" t="s">
+      <c r="J23" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24" s="3">
+        <v>17</v>
+      </c>
+      <c r="B24" s="11"/>
+      <c r="C24" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D24" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I24" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="J24" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="A25" s="3">
+        <v>18</v>
+      </c>
+      <c r="B25" s="11"/>
+      <c r="C25" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I25" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11">
+      <c r="A26" s="3">
+        <v>19</v>
+      </c>
+      <c r="B26" s="9"/>
+      <c r="C26" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I26" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="J26" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
+      <c r="A27" s="3">
+        <v>20</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I27" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K27" s="7" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <hyperlinks>
-    <hyperlink ref="D8" r:id="rId1" xr:uid="{96B02169-FF8B-4C6D-9861-B1FF6D9FFA44}"/>
-    <hyperlink ref="D9" r:id="rId2" xr:uid="{7EBF558B-AD84-48C4-BFD0-1B0FABBBDE93}"/>
-    <hyperlink ref="D10" r:id="rId3" xr:uid="{71D7476D-A843-4F5E-9D30-F45859B20076}"/>
-    <hyperlink ref="D11" r:id="rId4" xr:uid="{7566836C-A68A-46B1-92DD-C6EDA397B3DB}"/>
-    <hyperlink ref="D4" r:id="rId5" xr:uid="{7393101A-AB0A-4579-A972-F38C2C0EC13D}"/>
-    <hyperlink ref="D5:D7" r:id="rId6" display="gf180mcu_stdcells" xr:uid="{B9DE6BBC-0C69-4581-9249-E15DB0706FB4}"/>
-    <hyperlink ref="D12" r:id="rId7" xr:uid="{32280CC4-B8B0-4801-8042-3F259E8105B3}"/>
-    <hyperlink ref="D13" r:id="rId8" xr:uid="{C03EC173-0A90-4CFE-A545-060657B9C27D}"/>
-    <hyperlink ref="D16" r:id="rId9" xr:uid="{0D0DDB28-8942-43DD-834F-24F6CB67DF40}"/>
-    <hyperlink ref="D15" r:id="rId10" xr:uid="{FC2B0A46-C7C0-4FE4-8979-319B24915BCA}"/>
-    <hyperlink ref="D17" r:id="rId11" xr:uid="{DFD89CA2-3297-4298-B03D-55C8B623ABD0}"/>
-    <hyperlink ref="D18" r:id="rId12" xr:uid="{68F42C81-B341-4F88-8B82-EC45137B713A}"/>
-    <hyperlink ref="D19" r:id="rId13" xr:uid="{094BDAD3-A1C5-4C19-9C8D-107DFB2CA644}"/>
-    <hyperlink ref="D20" r:id="rId14" xr:uid="{75BB7E37-A25E-40CB-84D9-D881201AC00C}"/>
-    <hyperlink ref="D21" r:id="rId15" xr:uid="{D32F0983-8E06-499B-A5FC-5A07C4C61305}"/>
-    <hyperlink ref="D14" r:id="rId16" xr:uid="{DB6838D7-F735-4F3C-89CC-3FED158561A9}"/>
-    <hyperlink ref="D22" r:id="rId17" xr:uid="{DE0BC474-D7BF-4628-8E6C-E32B16E872E1}"/>
-    <hyperlink ref="D23" r:id="rId18" xr:uid="{E6411010-698F-4AEB-A056-0971ECB79120}"/>
+    <hyperlink ref="D12" r:id="rId1" xr:uid="{96B02169-FF8B-4C6D-9861-B1FF6D9FFA44}"/>
+    <hyperlink ref="D13" r:id="rId2" xr:uid="{7EBF558B-AD84-48C4-BFD0-1B0FABBBDE93}"/>
+    <hyperlink ref="D14" r:id="rId3" xr:uid="{71D7476D-A843-4F5E-9D30-F45859B20076}"/>
+    <hyperlink ref="D15" r:id="rId4" xr:uid="{7566836C-A68A-46B1-92DD-C6EDA397B3DB}"/>
+    <hyperlink ref="D8" r:id="rId5" xr:uid="{7393101A-AB0A-4579-A972-F38C2C0EC13D}"/>
+    <hyperlink ref="D9:D11" r:id="rId6" display="gf180mcu_stdcells" xr:uid="{B9DE6BBC-0C69-4581-9249-E15DB0706FB4}"/>
+    <hyperlink ref="D16" r:id="rId7" xr:uid="{32280CC4-B8B0-4801-8042-3F259E8105B3}"/>
+    <hyperlink ref="D17" r:id="rId8" xr:uid="{C03EC173-0A90-4CFE-A545-060657B9C27D}"/>
+    <hyperlink ref="D20" r:id="rId9" xr:uid="{0D0DDB28-8942-43DD-834F-24F6CB67DF40}"/>
+    <hyperlink ref="D19" r:id="rId10" xr:uid="{FC2B0A46-C7C0-4FE4-8979-319B24915BCA}"/>
+    <hyperlink ref="D21" r:id="rId11" xr:uid="{DFD89CA2-3297-4298-B03D-55C8B623ABD0}"/>
+    <hyperlink ref="D22" r:id="rId12" xr:uid="{68F42C81-B341-4F88-8B82-EC45137B713A}"/>
+    <hyperlink ref="D23" r:id="rId13" xr:uid="{094BDAD3-A1C5-4C19-9C8D-107DFB2CA644}"/>
+    <hyperlink ref="D24" r:id="rId14" xr:uid="{75BB7E37-A25E-40CB-84D9-D881201AC00C}"/>
+    <hyperlink ref="D25" r:id="rId15" xr:uid="{D32F0983-8E06-499B-A5FC-5A07C4C61305}"/>
+    <hyperlink ref="D18" r:id="rId16" xr:uid="{DB6838D7-F735-4F3C-89CC-3FED158561A9}"/>
+    <hyperlink ref="D26" r:id="rId17" xr:uid="{DE0BC474-D7BF-4628-8E6C-E32B16E872E1}"/>
+    <hyperlink ref="D27" r:id="rId18" xr:uid="{E6411010-698F-4AEB-A056-0971ECB79120}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId19"/>

</xml_diff>

<commit_message>
pfd lvs and drc passed
</commit_message>
<xml_diff>
--- a/review/project_status_tracker_super_long_wave.xlsx
+++ b/review/project_status_tracker_super_long_wave.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yutak\eda\designs\03_super_long_wave\2026_sscs_gf180\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5961A274-4B5D-475F-AF40-7CEFEB8665BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C94D15C-B4CF-472C-8654-709E6C5BF619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="status" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="68">
   <si>
     <t>No</t>
     <phoneticPr fontId="1"/>
@@ -280,10 +280,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>updated on Aug 3</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>GDS file is not created</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -293,6 +289,10 @@
   </si>
   <si>
     <t>GDS file was created, LVS and/or DRS are not passed.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>updated on Aug 4</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -841,17 +841,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K27"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
+  <dimension ref="A1:K26"/>
+  <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="5.75" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="18.125" customWidth="1"/>
+    <col min="3" max="3" width="18.08203125" customWidth="1"/>
     <col min="4" max="4" width="18.75" customWidth="1"/>
-    <col min="5" max="5" width="11.875" customWidth="1"/>
-    <col min="6" max="6" width="10.625" customWidth="1"/>
-    <col min="7" max="7" width="13.125" customWidth="1"/>
-    <col min="8" max="8" width="10.625" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="10.58203125" customWidth="1"/>
+    <col min="7" max="7" width="13.08203125" customWidth="1"/>
+    <col min="8" max="8" width="10.58203125" customWidth="1"/>
     <col min="9" max="9" width="12.25" customWidth="1"/>
     <col min="10" max="11" width="7.25" bestFit="1" customWidth="1"/>
   </cols>
@@ -866,100 +866,131 @@
     </row>
     <row r="2" spans="1:11">
       <c r="G2">
-        <f>COUNTIF(H8:H27,H2)</f>
-        <v>3</v>
+        <f>COUNTIF(H7:H26,H2)</f>
+        <v>2</v>
       </c>
       <c r="H2" s="22" t="s">
         <v>13</v>
       </c>
       <c r="I2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="G3">
-        <f t="shared" ref="G3:G4" si="0">COUNTIF(H9:H28,H3)</f>
+        <f>COUNTIF(H8:H27,H3)</f>
         <v>5</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>49</v>
       </c>
       <c r="I3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="G4">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <f>COUNTIF(H9:H28,H4)</f>
+        <v>11</v>
       </c>
       <c r="H4" s="18" t="s">
         <v>12</v>
       </c>
       <c r="I4" s="25" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E6" s="12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="14"/>
-      <c r="G6" s="19" t="s">
+      <c r="F5" s="14"/>
+      <c r="G5" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="13"/>
-    </row>
-    <row r="7" spans="1:11" s="1" customFormat="1" ht="42" customHeight="1">
-      <c r="A7" s="2" t="s">
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="13"/>
+    </row>
+    <row r="6" spans="1:11" s="1" customFormat="1" ht="42" customHeight="1">
+      <c r="A6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="F6" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="G6" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="H7" s="15" t="s">
+      <c r="H6" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="I7" s="15" t="s">
+      <c r="I6" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="J7" s="15" t="s">
+      <c r="J6" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="K7" s="15" t="s">
+      <c r="K6" s="15" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="3">
+        <v>1</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="3">
-        <v>1</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>42</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="B8" s="11"/>
       <c r="C8" s="4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D8" s="21" t="s">
         <v>50</v>
@@ -986,11 +1017,11 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>50</v>
@@ -1017,11 +1048,11 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="3">
-        <v>3</v>
-      </c>
-      <c r="B10" s="11"/>
+        <v>4</v>
+      </c>
+      <c r="B10" s="9"/>
       <c r="C10" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>50</v>
@@ -1048,14 +1079,16 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="3">
-        <v>4</v>
-      </c>
-      <c r="B11" s="9"/>
+        <v>5</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>5</v>
+      </c>
       <c r="C11" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>50</v>
+        <v>43</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>17</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>11</v>
@@ -1064,49 +1097,51 @@
         <v>12</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="J11" s="22" t="s">
+        <v>61</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="3">
-        <v>5</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>6</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F12" s="18" t="s">
         <v>12</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="I12" s="6">
         <v>1E-3</v>
       </c>
-      <c r="J12" s="22" t="s">
-        <v>61</v>
+      <c r="J12" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="K12" s="6" t="s">
         <v>48</v>
@@ -1114,51 +1149,49 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="3">
-        <v>6</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>10</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F13" s="18" t="s">
         <v>12</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I13" s="6">
-        <v>1E-3</v>
-      </c>
-      <c r="J13" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="K13" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I13" s="22">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J13" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="3">
-        <v>7</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>10</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="B14" s="9"/>
       <c r="C14" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>11</v>
@@ -1184,14 +1217,16 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="3">
-        <v>8</v>
-      </c>
-      <c r="B15" s="9"/>
+        <v>9</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>26</v>
+      </c>
       <c r="C15" s="4" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>11</v>
@@ -1199,34 +1234,34 @@
       <c r="F15" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G15" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I15" s="22">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="J15" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="K15" s="7" t="s">
-        <v>13</v>
+      <c r="G15" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I15" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>11</v>
@@ -1252,16 +1287,16 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="3">
-        <v>10</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>22</v>
+        <v>11</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>24</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>11</v>
@@ -1269,8 +1304,8 @@
       <c r="F17" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G17" s="24" t="s">
-        <v>11</v>
+      <c r="G17" s="23" t="s">
+        <v>46</v>
       </c>
       <c r="H17" s="22" t="s">
         <v>13</v>
@@ -1287,16 +1322,14 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="3">
-        <v>11</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>24</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B18" s="11"/>
       <c r="C18" s="4" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>11</v>
@@ -1322,11 +1355,11 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="3">
-        <v>12</v>
-      </c>
-      <c r="B19" s="11"/>
+        <v>13</v>
+      </c>
+      <c r="B19" s="9"/>
       <c r="C19" s="4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D19" s="16" t="s">
         <v>53</v>
@@ -1340,14 +1373,14 @@
       <c r="G19" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="H19" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="I19" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="J19" s="7" t="s">
-        <v>13</v>
+      <c r="H19" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I19" s="22">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="J19" s="22" t="s">
+        <v>61</v>
       </c>
       <c r="K19" s="7" t="s">
         <v>13</v>
@@ -1355,14 +1388,16 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="3">
-        <v>13</v>
-      </c>
-      <c r="B20" s="9"/>
+        <v>14</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>44</v>
+      </c>
       <c r="C20" s="4" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>11</v>
@@ -1370,34 +1405,34 @@
       <c r="F20" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G20" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I20" s="22">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="J20" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="K20" s="7" t="s">
-        <v>13</v>
+      <c r="G20" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I20" s="6">
+        <v>1E-3</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="3">
-        <v>14</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>44</v>
+        <v>15</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>25</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>11</v>
@@ -1423,13 +1458,11 @@
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="3">
-        <v>15</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>25</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="B22" s="11"/>
       <c r="C22" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>55</v>
@@ -1458,11 +1491,11 @@
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="3">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B23" s="11"/>
       <c r="C23" s="4" t="s">
-        <v>28</v>
+        <v>63</v>
       </c>
       <c r="D23" s="16" t="s">
         <v>55</v>
@@ -1491,11 +1524,11 @@
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="3">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B24" s="11"/>
       <c r="C24" s="4" t="s">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="D24" s="16" t="s">
         <v>55</v>
@@ -1524,14 +1557,14 @@
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="3">
-        <v>18</v>
-      </c>
-      <c r="B25" s="11"/>
+        <v>19</v>
+      </c>
+      <c r="B25" s="9"/>
       <c r="C25" s="4" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>11</v>
@@ -1557,14 +1590,16 @@
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="3">
-        <v>19</v>
-      </c>
-      <c r="B26" s="9"/>
+        <v>20</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="C26" s="4" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E26" s="10" t="s">
         <v>11</v>
@@ -1575,75 +1610,40 @@
       <c r="G26" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="H26" s="6" t="s">
-        <v>12</v>
+      <c r="H26" s="5" t="s">
+        <v>49</v>
       </c>
       <c r="I26" s="6">
         <v>1E-3</v>
       </c>
-      <c r="J26" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="K26" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11">
-      <c r="A27" s="3">
-        <v>20</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D27" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F27" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="G27" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="I27" s="6">
-        <v>1E-3</v>
-      </c>
-      <c r="J27" s="7" t="s">
+      <c r="J26" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="K27" s="7" t="s">
+      <c r="K26" s="7" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <hyperlinks>
-    <hyperlink ref="D12" r:id="rId1" xr:uid="{96B02169-FF8B-4C6D-9861-B1FF6D9FFA44}"/>
-    <hyperlink ref="D13" r:id="rId2" xr:uid="{7EBF558B-AD84-48C4-BFD0-1B0FABBBDE93}"/>
-    <hyperlink ref="D14" r:id="rId3" xr:uid="{71D7476D-A843-4F5E-9D30-F45859B20076}"/>
-    <hyperlink ref="D15" r:id="rId4" xr:uid="{7566836C-A68A-46B1-92DD-C6EDA397B3DB}"/>
-    <hyperlink ref="D8" r:id="rId5" xr:uid="{7393101A-AB0A-4579-A972-F38C2C0EC13D}"/>
-    <hyperlink ref="D9:D11" r:id="rId6" display="gf180mcu_stdcells" xr:uid="{B9DE6BBC-0C69-4581-9249-E15DB0706FB4}"/>
-    <hyperlink ref="D16" r:id="rId7" xr:uid="{32280CC4-B8B0-4801-8042-3F259E8105B3}"/>
-    <hyperlink ref="D17" r:id="rId8" xr:uid="{C03EC173-0A90-4CFE-A545-060657B9C27D}"/>
-    <hyperlink ref="D20" r:id="rId9" xr:uid="{0D0DDB28-8942-43DD-834F-24F6CB67DF40}"/>
-    <hyperlink ref="D19" r:id="rId10" xr:uid="{FC2B0A46-C7C0-4FE4-8979-319B24915BCA}"/>
-    <hyperlink ref="D21" r:id="rId11" xr:uid="{DFD89CA2-3297-4298-B03D-55C8B623ABD0}"/>
-    <hyperlink ref="D22" r:id="rId12" xr:uid="{68F42C81-B341-4F88-8B82-EC45137B713A}"/>
-    <hyperlink ref="D23" r:id="rId13" xr:uid="{094BDAD3-A1C5-4C19-9C8D-107DFB2CA644}"/>
-    <hyperlink ref="D24" r:id="rId14" xr:uid="{75BB7E37-A25E-40CB-84D9-D881201AC00C}"/>
-    <hyperlink ref="D25" r:id="rId15" xr:uid="{D32F0983-8E06-499B-A5FC-5A07C4C61305}"/>
-    <hyperlink ref="D18" r:id="rId16" xr:uid="{DB6838D7-F735-4F3C-89CC-3FED158561A9}"/>
-    <hyperlink ref="D26" r:id="rId17" xr:uid="{DE0BC474-D7BF-4628-8E6C-E32B16E872E1}"/>
-    <hyperlink ref="D27" r:id="rId18" xr:uid="{E6411010-698F-4AEB-A056-0971ECB79120}"/>
+    <hyperlink ref="D11" r:id="rId1" xr:uid="{96B02169-FF8B-4C6D-9861-B1FF6D9FFA44}"/>
+    <hyperlink ref="D12" r:id="rId2" xr:uid="{7EBF558B-AD84-48C4-BFD0-1B0FABBBDE93}"/>
+    <hyperlink ref="D13" r:id="rId3" xr:uid="{71D7476D-A843-4F5E-9D30-F45859B20076}"/>
+    <hyperlink ref="D14" r:id="rId4" xr:uid="{7566836C-A68A-46B1-92DD-C6EDA397B3DB}"/>
+    <hyperlink ref="D7" r:id="rId5" xr:uid="{7393101A-AB0A-4579-A972-F38C2C0EC13D}"/>
+    <hyperlink ref="D8:D10" r:id="rId6" display="gf180mcu_stdcells" xr:uid="{B9DE6BBC-0C69-4581-9249-E15DB0706FB4}"/>
+    <hyperlink ref="D15" r:id="rId7" xr:uid="{32280CC4-B8B0-4801-8042-3F259E8105B3}"/>
+    <hyperlink ref="D16" r:id="rId8" xr:uid="{C03EC173-0A90-4CFE-A545-060657B9C27D}"/>
+    <hyperlink ref="D19" r:id="rId9" xr:uid="{0D0DDB28-8942-43DD-834F-24F6CB67DF40}"/>
+    <hyperlink ref="D18" r:id="rId10" xr:uid="{FC2B0A46-C7C0-4FE4-8979-319B24915BCA}"/>
+    <hyperlink ref="D20" r:id="rId11" xr:uid="{DFD89CA2-3297-4298-B03D-55C8B623ABD0}"/>
+    <hyperlink ref="D21" r:id="rId12" xr:uid="{68F42C81-B341-4F88-8B82-EC45137B713A}"/>
+    <hyperlink ref="D22" r:id="rId13" xr:uid="{094BDAD3-A1C5-4C19-9C8D-107DFB2CA644}"/>
+    <hyperlink ref="D23" r:id="rId14" xr:uid="{75BB7E37-A25E-40CB-84D9-D881201AC00C}"/>
+    <hyperlink ref="D24" r:id="rId15" xr:uid="{D32F0983-8E06-499B-A5FC-5A07C4C61305}"/>
+    <hyperlink ref="D17" r:id="rId16" xr:uid="{DB6838D7-F735-4F3C-89CC-3FED158561A9}"/>
+    <hyperlink ref="D25" r:id="rId17" xr:uid="{DE0BC474-D7BF-4628-8E6C-E32B16E872E1}"/>
+    <hyperlink ref="D26" r:id="rId18" xr:uid="{E6411010-698F-4AEB-A056-0971ECB79120}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId19"/>

</xml_diff>

<commit_message>
ota_for_vco.gds lvs and drc passed
</commit_message>
<xml_diff>
--- a/review/project_status_tracker_super_long_wave.xlsx
+++ b/review/project_status_tracker_super_long_wave.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yutak\eda\designs\03_super_long_wave\2026_sscs_gf180\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C94D15C-B4CF-472C-8654-709E6C5BF619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EC78540-7E80-406C-8DB8-49A122313B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -879,7 +879,7 @@
     <row r="3" spans="1:11">
       <c r="G3">
         <f>COUNTIF(H8:H27,H3)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>49</v>
@@ -891,7 +891,7 @@
     <row r="4" spans="1:11">
       <c r="G4">
         <f>COUNTIF(H9:H28,H4)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H4" s="18" t="s">
         <v>12</v>
@@ -1099,14 +1099,14 @@
       <c r="G11" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="H11" s="5" t="s">
-        <v>49</v>
+      <c r="H11" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="I11" s="6">
         <v>1E-3</v>
       </c>
-      <c r="J11" s="22" t="s">
-        <v>61</v>
+      <c r="J11" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="K11" s="6" t="s">
         <v>48</v>

</xml_diff>